<commit_message>
Added voltmeters for testing mosfet voltages
</commit_message>
<xml_diff>
--- a/EE311_Charger_Parameters.xlsx
+++ b/EE311_Charger_Parameters.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kylep\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8deb8a6805bc7d3/Documents/311 Github/311/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F429902-05CA-41B1-BA41-8AC75F8D5DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="8_{2F429902-05CA-41B1-BA41-8AC75F8D5DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53D8691B-3200-4762-AB0E-7BF13A8B93DE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="64">
   <si>
     <t>Parameter</t>
   </si>
@@ -188,33 +188,18 @@
     <t>Vfb</t>
   </si>
   <si>
-    <t>Vopamp</t>
-  </si>
-  <si>
-    <t>Vsource</t>
-  </si>
-  <si>
-    <t>Vdrain</t>
-  </si>
-  <si>
     <t>Mpower</t>
   </si>
   <si>
     <t>Vrsense</t>
   </si>
   <si>
-    <t>Vbjt,base</t>
-  </si>
-  <si>
     <t>Rload</t>
   </si>
   <si>
     <t>VDS</t>
   </si>
   <si>
-    <t>VGS</t>
-  </si>
-  <si>
     <t>Evaluating Steady-State Operating Conditions (Simulation)</t>
   </si>
   <si>
@@ -236,18 +221,6 @@
     <t>Vfb = Vout × R7/(R6+R7)</t>
   </si>
   <si>
-    <t>Vopamp = Vgate (assumed 3.5 V)</t>
-  </si>
-  <si>
-    <t>Vsource = Vin - (Iout × Rsense)</t>
-  </si>
-  <si>
-    <t>Vdrain = Vout</t>
-  </si>
-  <si>
-    <t>VGS = Vgate - Vsource</t>
-  </si>
-  <si>
     <t>VDS = Vdrain - Vsource</t>
   </si>
   <si>
@@ -255,9 +228,6 @@
   </si>
   <si>
     <t>Vrsense = Iout × Rsense</t>
-  </si>
-  <si>
-    <t>Vbase = Vin - Vrsense</t>
   </si>
 </sst>
 </file>
@@ -268,7 +238,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -815,7 +785,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -832,9 +802,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="2" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -842,7 +809,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -850,21 +816,28 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -894,8 +867,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>231913</xdr:colOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>593670</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>44998</xdr:rowOff>
     </xdr:to>
@@ -1254,18 +1227,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AI58"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.44140625" customWidth="1"/>
     <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" customWidth="1"/>
+    <col min="25" max="25" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18">
+    <row r="3" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -1273,8 +1248,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1"/>
-    <row r="5" spans="1:7" ht="15.6" thickTop="1" thickBot="1">
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1285,8 +1260,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15" thickTop="1">
-      <c r="A6" s="22" t="s">
+    <row r="6" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="5">
@@ -1296,8 +1271,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="23" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="8">
@@ -1307,8 +1282,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="23" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="8">
@@ -1318,8 +1293,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="23" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="8">
@@ -1329,8 +1304,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="23" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
         <v>11</v>
       </c>
       <c r="B10" s="8">
@@ -1340,18 +1315,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="23" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="24">
+      <c r="B11" s="21">
         <v>0</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="22" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15" thickBot="1">
+    <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>18</v>
       </c>
@@ -1362,14 +1337,14 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15" thickTop="1"/>
-    <row r="18" spans="1:9" ht="18">
+    <row r="13" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="18" spans="1:9" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="15" thickBot="1"/>
-    <row r="20" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
+    <row r="19" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="20" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>0</v>
       </c>
@@ -1380,28 +1355,28 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15" thickTop="1">
-      <c r="A21" s="28" t="s">
+    <row r="21" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="30"/>
-    </row>
-    <row r="22" spans="1:9" ht="15" thickBot="1">
-      <c r="A22" s="31" t="s">
+      <c r="C21" s="26"/>
+    </row>
+    <row r="22" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="27" t="s">
         <v>23</v>
       </c>
       <c r="B22" s="11">
         <v>5</v>
       </c>
-      <c r="C22" s="32" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A23" s="31" t="s">
+      <c r="C22" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="27" t="s">
         <v>24</v>
       </c>
       <c r="B23" s="11">
@@ -1412,8 +1387,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A24" s="33" t="s">
+    <row r="24" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="29" t="s">
         <v>45</v>
       </c>
       <c r="B24" s="11">
@@ -1423,11 +1398,11 @@
       <c r="C24" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="H24" s="20"/>
-      <c r="I24" s="21"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A25" s="38" t="s">
+      <c r="H24" s="17"/>
+      <c r="I24" s="18"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="32" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="11">
@@ -1437,8 +1412,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A26" s="38" t="s">
+    <row r="26" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="32" t="s">
         <v>26</v>
       </c>
       <c r="B26" s="11">
@@ -1448,19 +1423,19 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A27" s="36" t="s">
+    <row r="27" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="30" t="s">
         <v>22</v>
       </c>
       <c r="B27" s="11">
         <v>0.5</v>
       </c>
-      <c r="C27" s="37" t="s">
+      <c r="C27" s="31" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A28" s="33" t="s">
+    <row r="28" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="29" t="s">
         <v>28</v>
       </c>
       <c r="B28" s="11">
@@ -1471,8 +1446,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A29" s="33" t="s">
+    <row r="29" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="29" t="s">
         <v>29</v>
       </c>
       <c r="B29" s="11">
@@ -1483,14 +1458,14 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15" thickTop="1"/>
-    <row r="35" spans="1:35" ht="18">
+    <row r="30" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="1:35" ht="18" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="1:35" ht="15" thickBot="1"/>
-    <row r="37" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
+    <row r="36" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="37" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>0</v>
       </c>
@@ -1501,28 +1476,28 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:35" ht="15" thickTop="1">
-      <c r="A38" s="28" t="s">
+    <row r="38" spans="1:35" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="29" t="s">
+      <c r="B38" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="C38" s="30"/>
-    </row>
-    <row r="39" spans="1:35" ht="15" thickBot="1">
-      <c r="A39" s="31" t="s">
+      <c r="C38" s="26"/>
+    </row>
+    <row r="39" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="27" t="s">
         <v>32</v>
       </c>
       <c r="B39" s="11">
         <v>5</v>
       </c>
-      <c r="C39" s="32" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A40" s="31" t="s">
+      <c r="C39" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="27" t="s">
         <v>8</v>
       </c>
       <c r="B40" s="11">
@@ -1532,8 +1507,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:35" ht="19.2" thickTop="1" thickBot="1">
-      <c r="A41" s="33" t="s">
+    <row r="41" spans="1:35" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="29" t="s">
         <v>46</v>
       </c>
       <c r="B41" s="11">
@@ -1546,11 +1521,11 @@
         <v>6</v>
       </c>
       <c r="Y41" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="42" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A42" s="38" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="42" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="32" t="s">
         <v>33</v>
       </c>
       <c r="B42" s="11">
@@ -1560,8 +1535,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A43" s="38" t="s">
+    <row r="43" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="32" t="s">
         <v>34</v>
       </c>
       <c r="B43" s="11">
@@ -1637,403 +1612,538 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="G44" s="40" t="s">
-        <v>60</v>
-      </c>
-      <c r="H44" s="41"/>
-      <c r="I44" s="41"/>
-      <c r="J44" s="42"/>
+    <row r="44" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G44" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="H44" s="35"/>
+      <c r="I44" s="35"/>
+      <c r="J44" s="36"/>
       <c r="L44" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M44" s="5">
-        <v>5</v>
-      </c>
-      <c r="N44" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O44" s="5">
-        <v>5</v>
-      </c>
-      <c r="P44" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q44" s="34">
-        <v>5</v>
-      </c>
-      <c r="R44" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S44" s="5">
-        <v>5</v>
-      </c>
-      <c r="T44" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U44" s="5">
-        <v>5</v>
-      </c>
-      <c r="V44" s="17" t="s">
+      <c r="M44" s="44">
+        <v>5</v>
+      </c>
+      <c r="N44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="O44" s="44">
+        <v>5</v>
+      </c>
+      <c r="P44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q44" s="46">
+        <v>5</v>
+      </c>
+      <c r="R44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="S44" s="44">
+        <v>5</v>
+      </c>
+      <c r="T44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="U44" s="44">
+        <v>5</v>
+      </c>
+      <c r="V44" s="47" t="s">
         <v>3</v>
       </c>
       <c r="Y44" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="Z44" s="5"/>
-      <c r="AA44" s="16"/>
-      <c r="AB44" s="5"/>
-      <c r="AC44" s="16"/>
-      <c r="AD44" s="34"/>
-      <c r="AE44" s="16"/>
-      <c r="AF44" s="5"/>
-      <c r="AG44" s="16"/>
-      <c r="AH44" s="5"/>
-      <c r="AI44" s="17"/>
-    </row>
-    <row r="45" spans="1:35" ht="15" thickTop="1">
-      <c r="G45" s="43" t="s">
-        <v>61</v>
-      </c>
-      <c r="H45" s="44"/>
-      <c r="I45" s="44"/>
-      <c r="J45" s="45"/>
-      <c r="L45" s="27" t="s">
+      <c r="Z44" s="44">
+        <v>5</v>
+      </c>
+      <c r="AA44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB44" s="44">
+        <v>5</v>
+      </c>
+      <c r="AC44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD44" s="46">
+        <v>5</v>
+      </c>
+      <c r="AE44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF44" s="44">
+        <v>5</v>
+      </c>
+      <c r="AG44" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH44" s="44">
+        <v>5</v>
+      </c>
+      <c r="AI44" s="47" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:35" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="G45" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="H45" s="42"/>
+      <c r="I45" s="42"/>
+      <c r="J45" s="38"/>
+      <c r="L45" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="M45" s="26">
+      <c r="M45" s="48">
         <f>M46*M47</f>
         <v>3.5000000000000004</v>
       </c>
-      <c r="N45" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O45" s="26">
+      <c r="N45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="O45" s="48">
         <f t="shared" ref="O45:U45" si="0">O46*O47</f>
-        <v>3.5</v>
-      </c>
-      <c r="P45" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q45" s="26">
+        <v>3.5000000000000004</v>
+      </c>
+      <c r="P45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q45" s="48">
         <f t="shared" si="0"/>
         <v>3.5</v>
       </c>
-      <c r="R45" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S45" s="26">
+      <c r="R45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="S45" s="48">
         <f t="shared" si="0"/>
-        <v>1.5</v>
-      </c>
-      <c r="T45" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U45" s="26">
+        <v>3.5</v>
+      </c>
+      <c r="T45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="U45" s="48">
         <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-      <c r="V45" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y45" s="27" t="s">
+        <v>2.5</v>
+      </c>
+      <c r="V45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y45" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="Z45" s="26"/>
-      <c r="AA45" s="16"/>
-      <c r="AB45" s="26"/>
-      <c r="AC45" s="16"/>
-      <c r="AD45" s="26"/>
-      <c r="AE45" s="16"/>
-      <c r="AF45" s="26"/>
-      <c r="AG45" s="16"/>
-      <c r="AH45" s="26"/>
-      <c r="AI45" s="16"/>
-    </row>
-    <row r="46" spans="1:35">
-      <c r="G46" s="43" t="s">
-        <v>62</v>
-      </c>
-      <c r="H46" s="44"/>
-      <c r="I46" s="44"/>
-      <c r="J46" s="45"/>
+      <c r="Z45" s="48">
+        <v>3.5110000000000001</v>
+      </c>
+      <c r="AA45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB45" s="48">
+        <v>3.484</v>
+      </c>
+      <c r="AC45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD45" s="48">
+        <v>3.4809999999999999</v>
+      </c>
+      <c r="AE45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF45" s="48">
+        <v>1.4219999999999999</v>
+      </c>
+      <c r="AG45" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH45" s="48">
+        <v>0.71299999999999997</v>
+      </c>
+      <c r="AI45" s="45" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="G46" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="H46" s="42"/>
+      <c r="I46" s="42"/>
+      <c r="J46" s="38"/>
       <c r="L46" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="M46" s="39">
+      <c r="M46" s="33">
         <f>MIN(3.5/M47,0.5)</f>
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="N46" s="37" t="s">
+      <c r="N46" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="O46" s="8">
+      <c r="O46" s="33">
         <f t="shared" ref="O46:U46" si="1">MIN(3.5/O47,0.5)</f>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="P46" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q46" s="33">
+        <f t="shared" si="1"/>
+        <v>0.11666666666666667</v>
+      </c>
+      <c r="R46" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="S46" s="33">
+        <f t="shared" si="1"/>
         <v>0.35</v>
       </c>
-      <c r="P46" s="37" t="s">
+      <c r="T46" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="Q46" s="8">
+      <c r="U46" s="33">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="R46" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="S46" s="8">
-        <f t="shared" si="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="T46" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="U46" s="8">
-        <f t="shared" si="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="V46" s="37" t="s">
+      <c r="V46" s="43" t="s">
         <v>10</v>
       </c>
       <c r="Y46" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="Z46" s="39"/>
-      <c r="AA46" s="37"/>
-      <c r="AB46" s="8"/>
-      <c r="AC46" s="37"/>
-      <c r="AD46" s="8"/>
-      <c r="AE46" s="37"/>
-      <c r="AF46" s="8"/>
-      <c r="AG46" s="37"/>
-      <c r="AH46" s="8"/>
-      <c r="AI46" s="37"/>
-    </row>
-    <row r="47" spans="1:35">
-      <c r="G47" s="43" t="s">
-        <v>63</v>
-      </c>
-      <c r="H47" s="44"/>
-      <c r="I47" s="44"/>
-      <c r="J47" s="45"/>
+      <c r="Z46" s="33">
+        <v>3.5110000000000002E-2</v>
+      </c>
+      <c r="AA46" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="AB46" s="33">
+        <v>6.9599999999999995E-2</v>
+      </c>
+      <c r="AC46" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD46" s="33">
+        <v>0.11600000000000001</v>
+      </c>
+      <c r="AE46" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF46" s="33">
+        <v>0.14219999999999999</v>
+      </c>
+      <c r="AG46" s="43" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH46" s="33">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="AI46" s="43" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="G47" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="H47" s="42"/>
+      <c r="I47" s="42"/>
+      <c r="J47" s="38"/>
       <c r="L47" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="M47" s="8">
+        <v>52</v>
+      </c>
+      <c r="M47" s="33">
         <v>100</v>
       </c>
-      <c r="N47" s="14" t="s">
+      <c r="N47" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="O47" s="8">
+      <c r="O47" s="33">
+        <v>50</v>
+      </c>
+      <c r="P47" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q47" s="50">
+        <v>30</v>
+      </c>
+      <c r="R47" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="S47" s="33">
         <v>10</v>
       </c>
-      <c r="P47" s="14" t="s">
+      <c r="T47" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="Q47" s="35">
-        <v>7</v>
-      </c>
-      <c r="R47" s="14" t="s">
+      <c r="U47" s="33">
+        <v>5</v>
+      </c>
+      <c r="V47" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="S47" s="8">
-        <v>3</v>
-      </c>
-      <c r="T47" s="14" t="s">
+      <c r="Y47" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="Z47" s="33">
+        <v>100</v>
+      </c>
+      <c r="AA47" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="U47" s="8">
-        <v>1</v>
-      </c>
-      <c r="V47" s="14" t="s">
+      <c r="AB47" s="33">
+        <v>50</v>
+      </c>
+      <c r="AC47" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="Y47" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z47" s="8"/>
-      <c r="AA47" s="14"/>
-      <c r="AB47" s="8"/>
-      <c r="AC47" s="14"/>
-      <c r="AD47" s="35"/>
-      <c r="AE47" s="14"/>
-      <c r="AF47" s="8"/>
-      <c r="AG47" s="14"/>
-      <c r="AH47" s="8"/>
-      <c r="AI47" s="14"/>
-    </row>
-    <row r="48" spans="1:35" ht="15" thickBot="1">
-      <c r="G48" s="43" t="s">
-        <v>64</v>
-      </c>
-      <c r="H48" s="44"/>
-      <c r="I48" s="44"/>
-      <c r="J48" s="45"/>
+      <c r="AD47" s="50">
+        <v>30</v>
+      </c>
+      <c r="AE47" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="AF47" s="33">
+        <v>10</v>
+      </c>
+      <c r="AG47" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH47" s="33">
+        <v>5</v>
+      </c>
+      <c r="AI47" s="49" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="48" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G48" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="H48" s="42"/>
+      <c r="I48" s="42"/>
+      <c r="J48" s="38"/>
       <c r="L48" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="M48" s="8">
+      <c r="M48" s="33">
         <v>1.75</v>
       </c>
-      <c r="N48" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="O48" s="8">
+      <c r="N48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="O48" s="33">
         <v>1.75</v>
       </c>
-      <c r="P48" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q48" s="35">
+      <c r="P48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q48" s="50">
         <v>1.75</v>
       </c>
-      <c r="R48" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="S48" s="8">
+      <c r="R48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="S48" s="33">
         <v>1.75</v>
       </c>
-      <c r="T48" s="18" t="s">
-        <v>3</v>
-      </c>
-      <c r="U48" s="8">
+      <c r="T48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="U48" s="33">
         <v>1.75</v>
       </c>
-      <c r="V48" s="18" t="s">
+      <c r="V48" s="51" t="s">
         <v>3</v>
       </c>
       <c r="Y48" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="Z48" s="8"/>
-      <c r="AA48" s="18"/>
-      <c r="AB48" s="8"/>
-      <c r="AC48" s="18"/>
-      <c r="AD48" s="35"/>
-      <c r="AE48" s="18"/>
-      <c r="AF48" s="8"/>
-      <c r="AG48" s="18"/>
-      <c r="AH48" s="8"/>
-      <c r="AI48" s="18"/>
-    </row>
-    <row r="49" spans="1:35" ht="19.2" thickTop="1" thickBot="1">
+      <c r="Z48" s="33">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AA48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB48" s="33">
+        <v>1.7511000000000001</v>
+      </c>
+      <c r="AC48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD48" s="50">
+        <v>1.7511000000000001</v>
+      </c>
+      <c r="AE48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF48" s="33">
+        <v>1.7511000000000001</v>
+      </c>
+      <c r="AG48" s="51" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH48" s="33">
+        <v>1.7511000000000001</v>
+      </c>
+      <c r="AI48" s="51" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:35" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G49" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="H49" s="44"/>
-      <c r="I49" s="44"/>
-      <c r="J49" s="45"/>
+      <c r="G49" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="H49" s="42"/>
+      <c r="I49" s="42"/>
+      <c r="J49" s="38"/>
       <c r="L49" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="M49" s="8">
+      <c r="M49" s="33">
         <f>M45/2</f>
         <v>1.7500000000000002</v>
       </c>
-      <c r="N49" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O49" s="8">
+      <c r="N49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="O49" s="33">
         <f t="shared" ref="O49:U49" si="2">O45/2</f>
-        <v>1.75</v>
-      </c>
-      <c r="P49" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q49" s="8">
+        <v>1.7500000000000002</v>
+      </c>
+      <c r="P49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q49" s="33">
         <f t="shared" si="2"/>
         <v>1.75</v>
       </c>
-      <c r="R49" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S49" s="8">
+      <c r="R49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="S49" s="33">
         <f t="shared" si="2"/>
-        <v>0.75</v>
-      </c>
-      <c r="T49" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U49" s="8">
+        <v>1.75</v>
+      </c>
+      <c r="T49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="U49" s="33">
         <f t="shared" si="2"/>
-        <v>0.25</v>
-      </c>
-      <c r="V49" s="16" t="s">
+        <v>1.25</v>
+      </c>
+      <c r="V49" s="45" t="s">
         <v>3</v>
       </c>
       <c r="Y49" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="Z49" s="8"/>
-      <c r="AA49" s="16"/>
-      <c r="AB49" s="8"/>
-      <c r="AC49" s="16"/>
-      <c r="AD49" s="8"/>
-      <c r="AE49" s="16"/>
-      <c r="AF49" s="8"/>
-      <c r="AG49" s="16"/>
-      <c r="AH49" s="8"/>
-      <c r="AI49" s="16"/>
-    </row>
-    <row r="50" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="G50" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="H50" s="44"/>
-      <c r="I50" s="44"/>
-      <c r="J50" s="45"/>
-      <c r="L50" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="M50" s="8">
-        <v>3.5</v>
-      </c>
-      <c r="N50" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O50" s="8">
-        <v>3.5</v>
-      </c>
-      <c r="P50" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q50" s="35">
-        <v>3.5</v>
-      </c>
-      <c r="R50" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S50" s="8">
-        <v>3.5</v>
-      </c>
-      <c r="T50" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U50" s="8">
-        <v>3.5</v>
-      </c>
-      <c r="V50" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y50" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="Z50" s="8"/>
-      <c r="AA50" s="16"/>
-      <c r="AB50" s="8"/>
-      <c r="AC50" s="16"/>
-      <c r="AD50" s="35"/>
-      <c r="AE50" s="16"/>
-      <c r="AF50" s="8"/>
-      <c r="AG50" s="16"/>
-      <c r="AH50" s="8"/>
-      <c r="AI50" s="16"/>
-    </row>
-    <row r="51" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
+      <c r="Z49" s="33">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AA49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB49" s="33">
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="AC49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD49" s="33">
+        <v>1.7511000000000001</v>
+      </c>
+      <c r="AE49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF49" s="33">
+        <v>0.71</v>
+      </c>
+      <c r="AG49" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH49" s="33">
+        <v>0.35099999999999998</v>
+      </c>
+      <c r="AI49" s="45" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G50" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="H50" s="42"/>
+      <c r="I50" s="42"/>
+      <c r="J50" s="38"/>
+      <c r="L50" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="M50" s="33">
+        <f>M45-M44+M52</f>
+        <v>-1.4509999999999996</v>
+      </c>
+      <c r="N50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="O50" s="33">
+        <f>O45-O44+O52</f>
+        <v>-1.4019999999999995</v>
+      </c>
+      <c r="P50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q50" s="33">
+        <f>Q45-Q44+Q52</f>
+        <v>-1.3366666666666667</v>
+      </c>
+      <c r="R50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="S50" s="33">
+        <f>S45-S44+S52</f>
+        <v>-1.01</v>
+      </c>
+      <c r="T50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="U50" s="33">
+        <f>U45-U44+U52</f>
+        <v>-1.8</v>
+      </c>
+      <c r="V50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y50" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z50" s="33"/>
+      <c r="AA50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB50" s="33"/>
+      <c r="AC50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD50" s="33"/>
+      <c r="AE50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF50" s="33"/>
+      <c r="AG50" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH50" s="33"/>
+      <c r="AI50" s="45" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
@@ -2043,407 +2153,199 @@
       <c r="C51" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G51" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="H51" s="44"/>
-      <c r="I51" s="44"/>
-      <c r="J51" s="45"/>
-      <c r="L51" s="23" t="s">
+      <c r="G51" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="H51" s="42"/>
+      <c r="I51" s="42"/>
+      <c r="J51" s="38"/>
+      <c r="L51" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M51" s="33">
+        <f>ABS(M50)*M46</f>
+        <v>5.078499999999999E-2</v>
+      </c>
+      <c r="N51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="O51" s="33">
+        <f>ABS(O50)*O46</f>
+        <v>9.8139999999999977E-2</v>
+      </c>
+      <c r="P51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q51" s="33">
+        <f>ABS(Q50)*Q46</f>
+        <v>0.15594444444444444</v>
+      </c>
+      <c r="R51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="S51" s="33">
+        <f>ABS(S50)*S46</f>
+        <v>0.35349999999999998</v>
+      </c>
+      <c r="T51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="U51" s="33">
+        <f>ABS(U50)*U46</f>
+        <v>0.9</v>
+      </c>
+      <c r="V51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="Y51" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="Z51" s="33"/>
+      <c r="AA51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB51" s="33"/>
+      <c r="AC51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD51" s="33"/>
+      <c r="AE51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF51" s="33"/>
+      <c r="AG51" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH51" s="33"/>
+      <c r="AI51" s="45" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:35" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B52" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C52" s="26"/>
+      <c r="G52" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H52" s="40"/>
+      <c r="I52" s="40"/>
+      <c r="J52" s="41"/>
+      <c r="L52" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="M51" s="8">
-        <f>M44-(M46*1.4)</f>
-        <v>4.9509999999999996</v>
-      </c>
-      <c r="N51" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O51" s="8">
-        <f t="shared" ref="O51:U51" si="3">O44-(O46*1.4)</f>
-        <v>4.51</v>
-      </c>
-      <c r="P51" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q51" s="8">
-        <f t="shared" si="3"/>
-        <v>4.3</v>
-      </c>
-      <c r="R51" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S51" s="8">
-        <f t="shared" si="3"/>
-        <v>4.3</v>
-      </c>
-      <c r="T51" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U51" s="8">
-        <f t="shared" si="3"/>
-        <v>4.3</v>
-      </c>
-      <c r="V51" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y51" s="23" t="s">
+      <c r="M52" s="33">
+        <f>M46*1.4</f>
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="N52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="O52" s="33">
+        <f>O46*1.4</f>
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="P52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q52" s="33">
+        <f>Q46*1.4</f>
+        <v>0.16333333333333333</v>
+      </c>
+      <c r="R52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="S52" s="33">
+        <f>S46*1.4</f>
+        <v>0.48999999999999994</v>
+      </c>
+      <c r="T52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="U52" s="33">
+        <f>U46*1.4</f>
+        <v>0.7</v>
+      </c>
+      <c r="V52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y52" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="Z51" s="8"/>
-      <c r="AA51" s="16"/>
-      <c r="AB51" s="8"/>
-      <c r="AC51" s="16"/>
-      <c r="AD51" s="8"/>
-      <c r="AE51" s="16"/>
-      <c r="AF51" s="8"/>
-      <c r="AG51" s="16"/>
-      <c r="AH51" s="8"/>
-      <c r="AI51" s="16"/>
-    </row>
-    <row r="52" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A52" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="B52" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="C52" s="30"/>
-      <c r="G52" s="43" t="s">
-        <v>68</v>
-      </c>
-      <c r="H52" s="44"/>
-      <c r="I52" s="44"/>
-      <c r="J52" s="45"/>
-      <c r="L52" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="M52" s="8">
-        <f>M45</f>
-        <v>3.5000000000000004</v>
-      </c>
-      <c r="N52" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O52" s="8">
-        <f t="shared" ref="O52:U52" si="4">O45</f>
-        <v>3.5</v>
-      </c>
-      <c r="P52" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q52" s="8">
-        <f t="shared" si="4"/>
-        <v>3.5</v>
-      </c>
-      <c r="R52" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S52" s="8">
-        <f t="shared" si="4"/>
-        <v>1.5</v>
-      </c>
-      <c r="T52" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U52" s="8">
-        <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-      <c r="V52" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y52" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="Z52" s="8"/>
-      <c r="AA52" s="16"/>
-      <c r="AB52" s="8"/>
-      <c r="AC52" s="16"/>
-      <c r="AD52" s="8"/>
-      <c r="AE52" s="16"/>
-      <c r="AF52" s="8"/>
-      <c r="AG52" s="16"/>
-      <c r="AH52" s="8"/>
-      <c r="AI52" s="16"/>
-    </row>
-    <row r="53" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A53" s="31" t="s">
+      <c r="Z52" s="33"/>
+      <c r="AA52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB52" s="33"/>
+      <c r="AC52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD52" s="33"/>
+      <c r="AE52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF52" s="33"/>
+      <c r="AG52" s="45" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH52" s="33"/>
+      <c r="AI52" s="45" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="27" t="s">
         <v>39</v>
       </c>
       <c r="B53" s="11">
         <f>B6</f>
         <v>5</v>
       </c>
-      <c r="C53" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="G53" s="43" t="s">
-        <v>69</v>
-      </c>
-      <c r="H53" s="44"/>
-      <c r="I53" s="44"/>
-      <c r="J53" s="45"/>
-      <c r="L53" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="M53" s="8">
-        <f>M50-M51</f>
-        <v>-1.4509999999999996</v>
-      </c>
-      <c r="N53" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O53" s="8">
-        <f t="shared" ref="N53:V53" si="5">O50-O51</f>
-        <v>-1.0099999999999998</v>
-      </c>
-      <c r="P53" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q53" s="8">
-        <f t="shared" si="5"/>
-        <v>-0.79999999999999982</v>
-      </c>
-      <c r="R53" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S53" s="8">
-        <f t="shared" si="5"/>
-        <v>-0.79999999999999982</v>
-      </c>
-      <c r="T53" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U53" s="8">
-        <f t="shared" si="5"/>
-        <v>-0.79999999999999982</v>
-      </c>
-      <c r="V53" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y53" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="Z53" s="8"/>
-      <c r="AA53" s="16"/>
-      <c r="AB53" s="8"/>
-      <c r="AC53" s="16"/>
-      <c r="AD53" s="8"/>
-      <c r="AE53" s="16"/>
-      <c r="AF53" s="8"/>
-      <c r="AG53" s="16"/>
-      <c r="AH53" s="8"/>
-      <c r="AI53" s="16"/>
-    </row>
-    <row r="54" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A54" s="31" t="s">
+      <c r="C53" s="28" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="27" t="s">
         <v>44</v>
       </c>
       <c r="B54" s="11">
         <f>(B56*B57)</f>
-        <v>0.70499999999999996</v>
+        <v>0.7</v>
       </c>
       <c r="C54" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G54" s="43" t="s">
-        <v>70</v>
-      </c>
-      <c r="H54" s="44"/>
-      <c r="I54" s="44"/>
-      <c r="J54" s="45"/>
-      <c r="L54" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="M54" s="8">
-        <f>M52-M51</f>
-        <v>-1.4509999999999992</v>
-      </c>
-      <c r="N54" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O54" s="8">
-        <f t="shared" ref="N54:V54" si="6">O52-O51</f>
-        <v>-1.0099999999999998</v>
-      </c>
-      <c r="P54" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q54" s="8">
-        <f t="shared" si="6"/>
-        <v>-0.79999999999999982</v>
-      </c>
-      <c r="R54" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S54" s="8">
-        <f t="shared" si="6"/>
-        <v>-2.8</v>
-      </c>
-      <c r="T54" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U54" s="8">
-        <f t="shared" si="6"/>
-        <v>-3.8</v>
-      </c>
-      <c r="V54" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y54" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="Z54" s="8"/>
-      <c r="AA54" s="16"/>
-      <c r="AB54" s="8"/>
-      <c r="AC54" s="16"/>
-      <c r="AD54" s="8"/>
-      <c r="AE54" s="16"/>
-      <c r="AF54" s="8"/>
-      <c r="AG54" s="16"/>
-      <c r="AH54" s="8"/>
-      <c r="AI54" s="16"/>
-    </row>
-    <row r="55" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A55" s="31" t="s">
+    </row>
+    <row r="55" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="27" t="s">
         <v>40</v>
       </c>
       <c r="B55" s="11">
         <f>ABS(B6-(B56*B27))</f>
-        <v>4.2949999999999999</v>
+        <v>4.3</v>
       </c>
       <c r="C55" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="G55" s="43" t="s">
-        <v>71</v>
-      </c>
-      <c r="H55" s="44"/>
-      <c r="I55" s="44"/>
-      <c r="J55" s="45"/>
-      <c r="L55" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="M55" s="8">
-        <f>ABS(M54*M46)</f>
-        <v>5.0784999999999976E-2</v>
-      </c>
-      <c r="N55" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="O55" s="8">
-        <f t="shared" ref="N55:U55" si="7">ABS(O54*O46)</f>
-        <v>0.35349999999999993</v>
-      </c>
-      <c r="P55" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q55" s="8">
-        <f t="shared" si="7"/>
-        <v>0.39999999999999991</v>
-      </c>
-      <c r="R55" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="S55" s="8">
-        <f t="shared" si="7"/>
+    </row>
+    <row r="56" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="B56" s="11">
         <v>1.4</v>
-      </c>
-      <c r="T55" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="U55" s="8">
-        <f t="shared" si="7"/>
-        <v>1.9</v>
-      </c>
-      <c r="V55" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="Y55" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z55" s="8"/>
-      <c r="AA55" s="14"/>
-      <c r="AB55" s="8"/>
-      <c r="AC55" s="14"/>
-      <c r="AD55" s="8"/>
-      <c r="AE55" s="14"/>
-      <c r="AF55" s="8"/>
-      <c r="AG55" s="14"/>
-      <c r="AH55" s="8"/>
-      <c r="AI55" s="14"/>
-    </row>
-    <row r="56" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A56" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="B56" s="11">
-        <v>1.41</v>
       </c>
       <c r="C56" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="G56" s="43" t="s">
-        <v>72</v>
-      </c>
-      <c r="H56" s="44"/>
-      <c r="I56" s="44"/>
-      <c r="J56" s="45"/>
-      <c r="L56" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="M56" s="8">
-        <f>M46*1.4</f>
-        <v>4.9000000000000002E-2</v>
-      </c>
-      <c r="N56" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O56" s="8">
-        <f t="shared" ref="O56:U56" si="8">O46*1.4</f>
-        <v>0.48999999999999994</v>
-      </c>
-      <c r="P56" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q56" s="8">
-        <f t="shared" si="8"/>
-        <v>0.7</v>
-      </c>
-      <c r="R56" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S56" s="8">
-        <f t="shared" si="8"/>
-        <v>0.7</v>
-      </c>
-      <c r="T56" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U56" s="8">
-        <f t="shared" si="8"/>
-        <v>0.7</v>
-      </c>
-      <c r="V56" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y56" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="Z56" s="8"/>
-      <c r="AA56" s="16"/>
-      <c r="AB56" s="8"/>
-      <c r="AC56" s="16"/>
-      <c r="AD56" s="8"/>
-      <c r="AE56" s="16"/>
-      <c r="AF56" s="8"/>
-      <c r="AG56" s="16"/>
-      <c r="AH56" s="8"/>
-      <c r="AI56" s="16"/>
-    </row>
-    <row r="57" spans="1:35" ht="15.6" thickTop="1" thickBot="1">
-      <c r="A57" s="38" t="s">
+    </row>
+    <row r="57" spans="1:35" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="32" t="s">
         <v>43</v>
       </c>
       <c r="B57" s="11">
@@ -2452,65 +2354,8 @@
       <c r="C57" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="G57" s="46" t="s">
-        <v>73</v>
-      </c>
-      <c r="H57" s="47"/>
-      <c r="I57" s="47"/>
-      <c r="J57" s="48"/>
-      <c r="L57" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="M57" s="8">
-        <f>M44-M56</f>
-        <v>4.9509999999999996</v>
-      </c>
-      <c r="N57" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="O57" s="8">
-        <f t="shared" ref="O57:U57" si="9">O44-O56</f>
-        <v>4.51</v>
-      </c>
-      <c r="P57" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q57" s="8">
-        <f t="shared" si="9"/>
-        <v>4.3</v>
-      </c>
-      <c r="R57" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="S57" s="8">
-        <f t="shared" si="9"/>
-        <v>4.3</v>
-      </c>
-      <c r="T57" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="U57" s="8">
-        <f t="shared" si="9"/>
-        <v>4.3</v>
-      </c>
-      <c r="V57" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y57" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="Z57" s="8"/>
-      <c r="AA57" s="16"/>
-      <c r="AB57" s="8"/>
-      <c r="AC57" s="16"/>
-      <c r="AD57" s="8"/>
-      <c r="AE57" s="16"/>
-      <c r="AF57" s="8"/>
-      <c r="AG57" s="16"/>
-      <c r="AH57" s="8"/>
-      <c r="AI57" s="16"/>
-    </row>
-    <row r="58" spans="1:35" ht="15" thickTop="1"/>
+    </row>
+    <row r="58" spans="1:35" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="44" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Fixed the charger just needs a breaker now
Fixed the charger just needs a breaker now
</commit_message>
<xml_diff>
--- a/EE311_Charger_Parameters.xlsx
+++ b/EE311_Charger_Parameters.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d8deb8a6805bc7d3/Documents/311 Github/311/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hpre798\Downloads\311-Group-9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="210" documentId="8_{2F429902-05CA-41B1-BA41-8AC75F8D5DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF2A65D2-3D3E-4EAE-9875-A822D2BA1170}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C5C26B-082A-4702-9DBF-333ED5865572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -102,9 +101,6 @@
     <t>Selected Mosfet</t>
   </si>
   <si>
-    <t>IRF9Z24N</t>
-  </si>
-  <si>
     <t>Max ID</t>
   </si>
   <si>
@@ -132,9 +128,6 @@
     <t>Evaluating Key Opamp Parameters (Theoretical)</t>
   </si>
   <si>
-    <t>LM358</t>
-  </si>
-  <si>
     <t>Supply Voltage</t>
   </si>
   <si>
@@ -229,6 +222,12 @@
   </si>
   <si>
     <t>Iout = Vout/Rload</t>
+  </si>
+  <si>
+    <t>IRF4905PBF</t>
+  </si>
+  <si>
+    <t>TLV9062</t>
   </si>
 </sst>
 </file>
@@ -239,7 +238,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -859,59 +858,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>183930</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>131379</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>595877</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>136526</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2405B264-014E-5439-C1D8-2D194DF6FDA5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4555404" y="2537695"/>
-          <a:ext cx="19051536" cy="10391073"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1235,52 +1181,52 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AF72"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.44140625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" style="2" customWidth="1"/>
-    <col min="3" max="6" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="28.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" style="2" customWidth="1"/>
+    <col min="3" max="6" width="8.85546875" style="2"/>
     <col min="7" max="7" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="2"/>
+    <col min="8" max="8" width="8.85546875" style="2"/>
     <col min="9" max="9" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" style="2"/>
+    <col min="10" max="10" width="8.85546875" style="2"/>
     <col min="11" max="11" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.77734375" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="2" customWidth="1"/>
     <col min="13" max="13" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.88671875" style="2"/>
+    <col min="14" max="14" width="8.85546875" style="2"/>
     <col min="15" max="15" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.88671875" style="2"/>
+    <col min="16" max="16" width="8.85546875" style="2"/>
     <col min="17" max="17" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="20" width="8.88671875" style="2"/>
+    <col min="18" max="20" width="8.85546875" style="2"/>
     <col min="21" max="21" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.88671875" style="2"/>
+    <col min="22" max="22" width="8.85546875" style="2"/>
     <col min="23" max="23" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.88671875" style="2"/>
-    <col min="25" max="25" width="10.5546875" style="2" customWidth="1"/>
-    <col min="26" max="26" width="8.88671875" style="2"/>
+    <col min="24" max="24" width="8.85546875" style="2"/>
+    <col min="25" max="25" width="10.5703125" style="2" customWidth="1"/>
+    <col min="26" max="26" width="8.85546875" style="2"/>
     <col min="27" max="27" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.88671875" style="2"/>
+    <col min="28" max="28" width="8.85546875" style="2"/>
     <col min="29" max="29" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.88671875" style="2"/>
+    <col min="30" max="30" width="8.85546875" style="2"/>
     <col min="31" max="31" width="9" style="2" bestFit="1" customWidth="1"/>
-    <col min="32" max="16384" width="8.88671875" style="2"/>
+    <col min="32" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="18.600000000000001" thickBot="1"/>
-    <row r="5" spans="1:7" ht="19.2" thickTop="1" thickBot="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:7" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1291,7 +1237,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="18.600000000000001" thickTop="1">
+    <row r="6" spans="1:7" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
@@ -1302,7 +1248,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>15</v>
       </c>
@@ -1313,7 +1259,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>16</v>
       </c>
@@ -1324,7 +1270,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>17</v>
       </c>
@@ -1335,7 +1281,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
@@ -1346,7 +1292,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
@@ -1357,7 +1303,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="18.600000000000001" thickBot="1">
+    <row r="12" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="12" t="s">
         <v>18</v>
       </c>
@@ -1368,14 +1314,14 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="18.600000000000001" thickTop="1"/>
-    <row r="18" spans="1:9">
+    <row r="13" spans="1:7" ht="19.5" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="18.600000000000001" thickBot="1"/>
-    <row r="20" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="20" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>0</v>
       </c>
@@ -1386,45 +1332,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="18.600000000000001" thickTop="1">
+    <row r="21" spans="1:9" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A21" s="15" t="s">
         <v>20</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="C21" s="17"/>
     </row>
-    <row r="22" spans="1:9" ht="18.600000000000001" thickBot="1">
+    <row r="22" spans="1:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="13">
+        <v>5</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="13">
-        <v>5</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
-      <c r="A23" s="18" t="s">
-        <v>24</v>
-      </c>
       <c r="B23" s="13">
-        <f>B6-(B27*0.62)</f>
-        <v>4.6900000000000004</v>
+        <f>B6-(B27*0.6)</f>
+        <v>4.7</v>
       </c>
       <c r="C23" s="20" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
+    <row r="24" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="21" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B24" s="13">
-        <f>B41</f>
-        <v>3.5</v>
+        <f>5</f>
+        <v>5</v>
       </c>
       <c r="C24" s="20" t="s">
         <v>3</v>
@@ -1432,9 +1378,9 @@
       <c r="H24" s="22"/>
       <c r="I24" s="23"/>
     </row>
-    <row r="25" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
+    <row r="25" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="13">
         <v>2.5</v>
@@ -1443,9 +1389,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
+    <row r="26" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="13">
         <v>3.5</v>
@@ -1454,9 +1400,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
+    <row r="27" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B27" s="13">
         <v>0.5</v>
@@ -1465,38 +1411,38 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
+    <row r="28" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="13">
         <f>ABS((B23-B25)*B27)</f>
-        <v>1.0950000000000002</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="C28" s="27" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="19.2" thickTop="1" thickBot="1">
+    <row r="29" spans="1:9" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="13">
         <f>ABS((B23-B26)*B27)</f>
-        <v>0.5950000000000002</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="C29" s="20" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="18.600000000000001" thickTop="1"/>
-    <row r="35" spans="1:3">
+    <row r="30" spans="1:9" ht="19.5" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="18.600000000000001" thickBot="1"/>
-    <row r="37" spans="1:3" ht="19.2" thickTop="1" thickBot="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="37" spans="1:3" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>0</v>
       </c>
@@ -1507,18 +1453,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="18.600000000000001" thickTop="1">
+    <row r="38" spans="1:3" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A38" s="15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="C38" s="17"/>
     </row>
-    <row r="39" spans="1:3" ht="18.600000000000001" thickBot="1">
+    <row r="39" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="18" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B39" s="13">
         <v>5</v>
@@ -1527,7 +1473,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="19.2" thickTop="1" thickBot="1">
+    <row r="40" spans="1:3" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="18" t="s">
         <v>8</v>
       </c>
@@ -1538,20 +1484,20 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="19.2" thickTop="1" thickBot="1">
+    <row r="41" spans="1:3" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B41" s="13">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="C41" s="20" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="19.2" thickTop="1" thickBot="1">
+    <row r="42" spans="1:3" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B42" s="13">
         <v>1.25</v>
@@ -1560,9 +1506,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="19.2" thickTop="1" thickBot="1">
+    <row r="43" spans="1:3" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B43" s="13">
         <v>1.75</v>
@@ -1571,14 +1517,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="18.600000000000001" thickTop="1"/>
-    <row r="49" spans="1:32">
+    <row r="44" spans="1:3" ht="19.5" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="49" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="50" spans="1:32" ht="18.600000000000001" thickBot="1"/>
-    <row r="51" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" spans="1:32" ht="19.5" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="51" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
@@ -1589,18 +1535,18 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:32" ht="18.600000000000001" thickTop="1">
+    <row r="52" spans="1:32" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A52" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B52" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C52" s="17"/>
+    </row>
+    <row r="53" spans="1:32" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="18" t="s">
         <v>37</v>
-      </c>
-      <c r="B52" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="C52" s="17"/>
-    </row>
-    <row r="53" spans="1:32" ht="18.600000000000001" thickBot="1">
-      <c r="A53" s="18" t="s">
-        <v>39</v>
       </c>
       <c r="B53" s="13">
         <f>B6</f>
@@ -1610,43 +1556,43 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+    <row r="54" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="18" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B54" s="13">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="C54" s="20" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+    <row r="55" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="18" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B55" s="13">
         <f>ABS(B6-(B56*B27))</f>
-        <v>4.6900000000000004</v>
+        <v>4.7</v>
       </c>
       <c r="C55" s="20" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+    <row r="56" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B56" s="13">
+        <v>0.6</v>
+      </c>
+      <c r="C56" s="20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="57" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="12" t="s">
         <v>41</v>
-      </c>
-      <c r="B56" s="13">
-        <v>0.62</v>
-      </c>
-      <c r="C56" s="20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="57" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
-      <c r="A57" s="12" t="s">
-        <v>43</v>
       </c>
       <c r="B57" s="13">
         <v>0.5</v>
@@ -1655,17 +1601,17 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:32" ht="18.600000000000001" thickTop="1"/>
-    <row r="61" spans="1:32">
+    <row r="58" spans="1:32" ht="19.5" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:32" x14ac:dyDescent="0.3">
       <c r="F61" s="1" t="s">
         <v>6</v>
       </c>
       <c r="T61" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="62" spans="1:32" ht="18.600000000000001" thickBot="1"/>
-    <row r="63" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="62" spans="1:32" ht="19.5" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="63" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="F63" s="3" t="s">
         <v>0</v>
       </c>
@@ -1745,9 +1691,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+    <row r="64" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="28" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B64" s="29"/>
       <c r="C64" s="29"/>
@@ -1831,9 +1777,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="65" spans="1:32" ht="18.600000000000001" thickTop="1">
+    <row r="65" spans="1:32" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A65" s="35" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B65" s="36"/>
       <c r="C65" s="36"/>
@@ -1905,34 +1851,33 @@
         <v>3</v>
       </c>
       <c r="AA65" s="39">
-        <v>3.4929999999999999</v>
+        <v>3.45</v>
       </c>
       <c r="AB65" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AC65" s="39">
-        <v>2.4975000000000001</v>
+        <v>2.4660000000000002</v>
       </c>
       <c r="AD65" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AE65" s="39">
-        <f t="shared" ref="AE65" si="2">AE66*AE67</f>
-        <v>0.5</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="AF65" s="32" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:32">
+    <row r="66" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A66" s="35" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B66" s="36"/>
       <c r="C66" s="36"/>
       <c r="D66" s="37"/>
       <c r="F66" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G66" s="40">
         <f>MIN(3.5/G67,0.5)</f>
@@ -1942,42 +1887,42 @@
         <v>10</v>
       </c>
       <c r="I66" s="40">
-        <f t="shared" ref="I66:Q66" si="3">MIN(3.5/I67,0.5)</f>
+        <f t="shared" ref="I66:Q66" si="2">MIN(3.5/I67,0.5)</f>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="J66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="K66" s="40">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.11666666666666667</v>
       </c>
       <c r="L66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="M66" s="40">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="N66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="O66" s="40">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="P66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="Q66" s="40">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0.5</v>
       </c>
       <c r="R66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="T66" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="U66" s="40">
         <v>3.5110000000000002E-2</v>
@@ -1992,120 +1937,119 @@
         <v>10</v>
       </c>
       <c r="Y66" s="40">
-        <v>0.11990000000000001</v>
+        <v>0.11700000000000001</v>
       </c>
       <c r="Z66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="AA66" s="40">
-        <v>0.499</v>
+        <v>0.49199999999999999</v>
       </c>
       <c r="AB66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="AC66" s="40">
-        <v>0.4995</v>
+        <v>0.49299999999999999</v>
       </c>
       <c r="AD66" s="41" t="s">
         <v>10</v>
       </c>
       <c r="AE66" s="40">
-        <f t="shared" ref="AE66" si="4">MIN(3.5/AE67,0.5)</f>
-        <v>0.5</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="AF66" s="41" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="67" spans="1:32">
+    <row r="67" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A67" s="35" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B67" s="36"/>
       <c r="C67" s="36"/>
       <c r="D67" s="37"/>
       <c r="F67" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G67" s="40">
         <v>100</v>
       </c>
       <c r="H67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I67" s="40">
         <v>50</v>
       </c>
       <c r="J67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K67" s="43">
         <v>30</v>
       </c>
       <c r="L67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="M67" s="40">
         <v>7</v>
       </c>
       <c r="N67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="O67" s="40">
         <v>5</v>
       </c>
       <c r="P67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Q67" s="40">
         <v>1</v>
       </c>
       <c r="R67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="T67" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="U67" s="40">
         <v>100</v>
       </c>
       <c r="V67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="W67" s="40">
         <v>50</v>
       </c>
       <c r="X67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="Y67" s="43">
         <v>30</v>
       </c>
       <c r="Z67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AA67" s="40">
         <v>7</v>
       </c>
       <c r="AB67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AC67" s="40">
         <v>5</v>
       </c>
       <c r="AD67" s="42" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="AE67" s="40">
         <v>1</v>
       </c>
       <c r="AF67" s="42" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="68" spans="1:32" ht="18.600000000000001" thickBot="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="68" spans="1:32" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="35" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B68" s="36"/>
       <c r="C68" s="36"/>
@@ -2189,15 +2133,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+    <row r="69" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="35" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B69" s="36"/>
       <c r="C69" s="36"/>
       <c r="D69" s="37"/>
       <c r="F69" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G69" s="40">
         <f>G65/2</f>
@@ -2207,45 +2151,45 @@
         <v>3</v>
       </c>
       <c r="I69" s="40">
-        <f t="shared" ref="I69:O69" si="5">I65/2</f>
+        <f t="shared" ref="I69:O69" si="3">I65/2</f>
         <v>1.7500000000000002</v>
       </c>
       <c r="J69" s="32" t="s">
         <v>3</v>
       </c>
       <c r="K69" s="40">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>1.75</v>
       </c>
       <c r="L69" s="32" t="s">
         <v>3</v>
       </c>
       <c r="M69" s="40">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>1.75</v>
       </c>
       <c r="N69" s="32" t="s">
         <v>3</v>
       </c>
       <c r="O69" s="40">
-        <f t="shared" si="5"/>
+        <f t="shared" si="3"/>
         <v>1.25</v>
       </c>
       <c r="P69" s="32" t="s">
         <v>3</v>
       </c>
       <c r="Q69" s="40">
-        <f t="shared" ref="Q69" si="6">Q65/2</f>
+        <f t="shared" ref="Q69" si="4">Q65/2</f>
         <v>0.25</v>
       </c>
       <c r="R69" s="32" t="s">
         <v>3</v>
       </c>
       <c r="T69" s="7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="U69" s="40">
-        <v>1.77</v>
+        <v>1.7549999999999999</v>
       </c>
       <c r="V69" s="32" t="s">
         <v>3</v>
@@ -2263,307 +2207,307 @@
         <v>3</v>
       </c>
       <c r="AA69" s="40">
-        <v>1.7465999999999999</v>
+        <v>1.7250000000000001</v>
       </c>
       <c r="AB69" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AC69" s="40">
-        <v>1.24885</v>
+        <v>1.2330000000000001</v>
       </c>
       <c r="AD69" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AE69" s="40">
-        <v>0.25</v>
+        <v>0.247</v>
       </c>
       <c r="AF69" s="32" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+    <row r="70" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="35" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B70" s="36"/>
       <c r="C70" s="36"/>
       <c r="D70" s="37"/>
       <c r="F70" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G70" s="40">
         <f>G65-G64+G72</f>
-        <v>-1.4782999999999995</v>
+        <v>-1.4789999999999996</v>
       </c>
       <c r="H70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="I70" s="40">
         <f>I65-I64+I72</f>
-        <v>-1.4565999999999995</v>
+        <v>-1.4579999999999995</v>
       </c>
       <c r="J70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="K70" s="40">
         <f>K65-K64+K72</f>
-        <v>-1.4276666666666666</v>
+        <v>-1.43</v>
       </c>
       <c r="L70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="M70" s="40">
         <f>M65-M64+M72</f>
-        <v>-1.19</v>
+        <v>-1.2</v>
       </c>
       <c r="N70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="O70" s="40">
         <f>O65-O64+O72</f>
-        <v>-2.19</v>
+        <v>-2.2000000000000002</v>
       </c>
       <c r="P70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="Q70" s="40">
         <f>Q65-Q64+Q72</f>
-        <v>-4.1900000000000004</v>
+        <v>-4.2</v>
       </c>
       <c r="R70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="T70" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="U70" s="40">
+        <v>-1.466</v>
+      </c>
+      <c r="V70" s="32" t="s">
+        <v>3</v>
+      </c>
+      <c r="W70" s="40">
         <v>-1.44</v>
       </c>
-      <c r="V70" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="W70" s="40">
-        <v>-1.42</v>
-      </c>
       <c r="X70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="Y70" s="40">
-        <v>-1.4</v>
+        <v>-1.4179999999999999</v>
       </c>
       <c r="Z70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AA70" s="40">
-        <v>-1.1969000000000001</v>
+        <v>-1.25</v>
       </c>
       <c r="AB70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AC70" s="40">
-        <v>-2.19</v>
+        <v>-2.23</v>
       </c>
       <c r="AD70" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AE70" s="40">
-        <v>-4.18</v>
+        <v>-4.2</v>
       </c>
       <c r="AF70" s="32" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:32" ht="19.2" thickTop="1" thickBot="1">
+    <row r="71" spans="1:32" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A71" s="35" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B71" s="36"/>
       <c r="C71" s="36"/>
       <c r="D71" s="37"/>
       <c r="F71" s="45" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G71" s="40">
         <f>ABS(G70)*G66</f>
-        <v>5.1740499999999988E-2</v>
+        <v>5.1764999999999992E-2</v>
       </c>
       <c r="H71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="I71" s="40">
         <f>ABS(I70)*I66</f>
-        <v>0.10196199999999997</v>
+        <v>0.10205999999999997</v>
       </c>
       <c r="J71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="K71" s="40">
         <f>ABS(K70)*K66</f>
-        <v>0.1665611111111111</v>
+        <v>0.16683333333333333</v>
       </c>
       <c r="L71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="M71" s="40">
         <f>ABS(M70)*M66</f>
-        <v>0.59499999999999997</v>
+        <v>0.6</v>
       </c>
       <c r="N71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="O71" s="40">
         <f>ABS(O70)*O66</f>
-        <v>1.095</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="P71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="Q71" s="40">
         <f>ABS(Q70)*Q66</f>
-        <v>2.0950000000000002</v>
+        <v>2.1</v>
       </c>
       <c r="R71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="T71" s="45" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="U71" s="40">
         <f>ABS(U70*U66)</f>
-        <v>5.0558400000000003E-2</v>
+        <v>5.1471260000000005E-2</v>
       </c>
       <c r="V71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="W71" s="40">
-        <f t="shared" ref="W71:AE71" si="7">ABS(W70*W66)</f>
-        <v>9.8831999999999989E-2</v>
+        <f t="shared" ref="W71:AE71" si="5">ABS(W70*W66)</f>
+        <v>0.10022399999999999</v>
       </c>
       <c r="X71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="Y71" s="40">
-        <f t="shared" si="7"/>
-        <v>0.16786000000000001</v>
+        <f t="shared" si="5"/>
+        <v>0.165906</v>
       </c>
       <c r="Z71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="AA71" s="40">
-        <f t="shared" si="7"/>
-        <v>0.59725309999999998</v>
+        <f t="shared" si="5"/>
+        <v>0.61499999999999999</v>
       </c>
       <c r="AB71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="AC71" s="40">
-        <f t="shared" si="7"/>
-        <v>1.0939049999999999</v>
+        <f t="shared" si="5"/>
+        <v>1.0993899999999999</v>
       </c>
       <c r="AD71" s="32" t="s">
         <v>4</v>
       </c>
       <c r="AE71" s="40">
-        <f t="shared" si="7"/>
-        <v>2.09</v>
+        <f t="shared" si="5"/>
+        <v>2.0748000000000002</v>
       </c>
       <c r="AF71" s="32" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:32" ht="18.600000000000001" thickTop="1">
+    <row r="72" spans="1:32" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A72" s="46" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B72" s="47"/>
       <c r="C72" s="47"/>
       <c r="D72" s="48"/>
       <c r="F72" s="45" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G72" s="40">
-        <f>G66*0.62</f>
-        <v>2.1700000000000001E-2</v>
+        <f>G66*0.6</f>
+        <v>2.1000000000000001E-2</v>
       </c>
       <c r="H72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="I72" s="40">
-        <f>I66*0.62</f>
-        <v>4.3400000000000001E-2</v>
+        <f>I66*0.6</f>
+        <v>4.2000000000000003E-2</v>
       </c>
       <c r="J72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="K72" s="40">
-        <f>K66*0.62</f>
-        <v>7.2333333333333333E-2</v>
+        <f>K66*0.6</f>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="L72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="M72" s="40">
-        <f>M66*0.62</f>
-        <v>0.31</v>
+        <f>M66*0.6</f>
+        <v>0.3</v>
       </c>
       <c r="N72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="O72" s="40">
-        <f>O66*0.62</f>
-        <v>0.31</v>
+        <f>O66*0.6</f>
+        <v>0.3</v>
       </c>
       <c r="P72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="Q72" s="40">
-        <f>Q66*0.62</f>
-        <v>0.31</v>
+        <f>Q66*0.6</f>
+        <v>0.3</v>
       </c>
       <c r="R72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="T72" s="45" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="U72" s="40">
-        <f>0.62*U66</f>
-        <v>2.1768200000000001E-2</v>
+        <f>0.6*U66</f>
+        <v>2.1066000000000001E-2</v>
       </c>
       <c r="V72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="W72" s="40">
-        <f t="shared" ref="W72:AE72" si="8">0.62*W66</f>
-        <v>4.3151999999999996E-2</v>
+        <f>0.6*W66</f>
+        <v>4.1759999999999999E-2</v>
       </c>
       <c r="X72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="Y72" s="40">
-        <f t="shared" si="8"/>
-        <v>7.4338000000000001E-2</v>
+        <f>0.6*Y66</f>
+        <v>7.0199999999999999E-2</v>
       </c>
       <c r="Z72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AA72" s="40">
-        <f t="shared" si="8"/>
-        <v>0.30937999999999999</v>
+        <f>0.6*AA66</f>
+        <v>0.29519999999999996</v>
       </c>
       <c r="AB72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AC72" s="40">
-        <f t="shared" si="8"/>
-        <v>0.30969000000000002</v>
+        <f>0.6*AC66</f>
+        <v>0.29580000000000001</v>
       </c>
       <c r="AD72" s="32" t="s">
         <v>3</v>
       </c>
       <c r="AE72" s="40">
-        <f t="shared" si="8"/>
-        <v>0.31</v>
+        <f>0.6*AE66</f>
+        <v>0.2964</v>
       </c>
       <c r="AF72" s="32" t="s">
         <v>3</v>
@@ -2572,7 +2516,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="34" orientation="landscape" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>